<commit_message>
add insulated floor joists
</commit_message>
<xml_diff>
--- a/src/cubes/data/materials/materials.xlsx
+++ b/src/cubes/data/materials/materials.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/elizabeth-homes/src/cubes/data/materials/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hannes/Work/CUBES/src/cubes/data/materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3BFBE6E-E950-9A49-AF5C-57CFBE959AE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE9E57AC-A472-FD41-88AE-25F4B49D6A92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="860" yWindow="2300" windowWidth="26660" windowHeight="15800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="560" yWindow="-15760" windowWidth="26660" windowHeight="15800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="100">
   <si>
     <t>Material</t>
   </si>
@@ -333,6 +333,9 @@
   </si>
   <si>
     <t>Joists_with_100mm_insulation_CODE</t>
+  </si>
+  <si>
+    <t>Floor_joists_with_120mm_insulation_CODE</t>
   </si>
 </sst>
 </file>
@@ -711,10 +714,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K89"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="34.33203125" customWidth="1"/>
+    <col min="1" max="1" width="40" customWidth="1"/>
     <col min="2" max="5" width="20.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
     <col min="7" max="7" width="22.6640625" customWidth="1"/>
@@ -3740,6 +3743,38 @@
         <v>0</v>
       </c>
     </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>99</v>
+      </c>
+      <c r="B89">
+        <v>4.2999999999999997E-2</v>
+      </c>
+      <c r="D89">
+        <v>71</v>
+      </c>
+      <c r="E89">
+        <v>170</v>
+      </c>
+      <c r="F89" t="s">
+        <v>47</v>
+      </c>
+      <c r="G89">
+        <v>0.9</v>
+      </c>
+      <c r="H89">
+        <v>0.7</v>
+      </c>
+      <c r="I89">
+        <v>0.7</v>
+      </c>
+      <c r="J89" t="b">
+        <v>0</v>
+      </c>
+      <c r="K89" t="b">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>